<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.002-02 La mer dans la coquille
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.002-02.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.002-02.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La mer dans la poche</t>
+          <t>La mer dans la coquille</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>port, caisses mouillées, ponton, coquille</t>
+          <t>entrée, classe, puis maison, grains de sable sur le paillasson, seau en fer, bottes, odeur de bord de mer</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nino, papa</t>
+          <t>Nino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut faire écouter la mer dans sa coquille. Il parle trop tôt. Les mouettes couvrent sa voix. Il lève la main, il attend, puis papa l'entend.</t>
+          <t>Le paillasson gratte. Sur le fer, un éclat de seau luit. Nino veut parler de la mer dans la coquille, maintenant. Les mots se cognent à la classe. À la maison, près du seau, il parle trop vite. Il refuse de foncer, lève la main, attend. Merci vécu. Un éclat de seau reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une coquille grince dans la poche de Nino. Le bois du ponton est sombre, encore mouillé. Ça sent le sel et les caisses de poisson. Une écaille brille près d'une corde. Les mouettes crient, très haut. Tu as vu l'eau, Nino ? Elle tape le bois. Elle est verte, ce soir. Nino sort la coquille, toute rêche. Je veux que tu écoutes. La mer est dedans. On l'écoute, alors. En ce moment, papa compte des caisses. Il parle vers le bout du ponton. Sa voix se mêle aux mouettes. Papa, écoute ! Hush, hush ! Les mots tombent dans les cris. Personne ne se tourne. La coquille reste froide dans la paume. Papa. Papa compte encore, un doigt en l'air. Nino ferme la bouche. Il lève la main, tout droit. La coquille est dans l'autre main. Sa main reste en l'air, près de la corde. Une mouette passe, puis s'éloigne. Papa se tourne. Tu voulais dire quelque chose ? La mer. Dans la coquille. Je t'entends, maintenant. Papa se baisse. L'oreille touche le bord rêche. Hush. Hush, oui. Merci, Nino. Tu as attendu, et je t'ai entendu. L'eau tape encore le ponton, tout bas. La coquille garde le même hush. On la remet dans la poche ? Pour ce soir.</t>
+          <t>Le paillasson gratte sous les pieds. Des grains de sable restent dans les fibres. Ils piquent un peu, très fins. Un seau en fer est près des bottes. Sur le fer, un éclat de seau luit. Il brille, papa. Tu le vois, sur le seau ? Le seau sent le bord de mer. Les bottes sont rêches, un peu salées. Ça sent la mer. Tes mains sont froides, Nino. Je veux entendre la mer. Dans une coquille. On va à l'école. Le cartable est près de la porte. Oui, maman. Papa aide Nino à passer les bras. Le manteau sent un peu le sel. Je reviens te chercher. Oui, papa. Papa serre l'épaule de Nino. Ils poussent la porte de l'école. La classe sent les feuilles. Un tapis de laine attend sous la fenêtre. Bonjour. Bonjour, maîtresse. Nino pose le cartable près du tapis. Il s'assoit, le dos droit. La maîtresse pose une boîte sur la table. Elle ouvre le couvercle, sans un mot. Une coquille crème apparaît. Elle a des lignes, un peu rêche. La mer est dedans ! Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le dis, maintenant ! En ce moment, Nino ouvre la bouche. Ses mots se cognent à la classe. Un camarade parle près de la boîte. Personne ne tourne la tête. Oh. Le sourire de Nino disparaît. Ses épaules tombent un peu. Nino referme la bouche. Les mains restent sur les genoux. À la sortie, papa attend près de la porte. On rentre, Nino ? Oui. Le soir, le paillasson gratte de nouveau. Nino touche l'éclat de seau, un instant. Te voilà, Nino. Les bottes sont là. J'ai quelque chose, maintenant ! Nino avance trop vite vers le seau. Maman accroche le manteau.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une coquille grince dans la poche de Nino. Le bois du ponton est sombre, encore mouillé. Ça sent le sel et les caisses de poisson. Une écaille brille près d'une corde. Les mouettes crient, très haut. Tu as vu l'eau, Nino ? Elle tape le bois. Elle est verte, ce soir. Nino sort la coquille, toute rêche. Je veux que tu écoutes. La mer est dedans. On l'écoute, alors. En ce moment, papa compte des caisses. Il parle vers le bout du ponton. Sa voix se mêle aux mouettes. Papa, écoute ! Hush, hush ! Les mots tombent dans les cris. Personne ne se tourne. La coquille reste froide dans la paume. Papa. Papa compte encore, un doigt en l'air. Nino ferme la bouche. Il lève la main, tout droit. La coquille est dans l'autre main. Sa main reste en l'air, près de la corde. Une mouette passe, puis s'éloigne. Papa se tourne. Tu voulais dire quelque chose ? La mer. Dans la coquille. Je t'entends, maintenant. Papa se baisse. L'oreille touche le bord rêche. Hush. Hush, oui. Merci, Nino. Tu as attendu, et je t'ai entendu. L'eau tape encore le ponton, tout bas. La coquille garde le même hush. On la remet dans la poche ? Pour ce soir.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le paillasson gratte sous les pieds. Des grains de sable restent dans les fibres. Ils piquent un peu, très fins. Un seau en fer est près des bottes. Sur le fer, un &lt;emphasis level="moderate"&gt;éclat de seau&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le seau ? Le seau sent le bord de mer. Les bottes sont rêches, un peu salées. Ça sent la mer. Tes mains sont froides, Nino. Je veux entendre la mer. Dans une coquille. On va à l'école. Le cartable est près de la porte. Oui, maman. Papa aide Nino à passer les bras. Le manteau sent un peu le sel. Je reviens te chercher. Oui, papa. Papa serre l'épaule de Nino. Ils poussent la porte de l'école. La classe sent les feuilles. Un tapis de laine attend sous la fenêtre. Bonjour. Bonjour, maîtresse. Nino pose le cartable près du tapis. Il s'assoit, le dos droit. La maîtresse pose une boîte sur la table. Elle ouvre le couvercle, sans un mot. Une coquille crème apparaît. Elle a des lignes, un peu rêche. La mer est dedans ! Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le dis, maintenant ! En ce moment, Nino ouvre la bouche. Ses mots se cognent à la classe. Un camarade parle près de la boîte. Personne ne tourne la tête. Oh. Le sourire de Nino disparaît. Ses épaules tombent un peu. Nino referme la bouche. Les mains restent sur les genoux. À la sortie, papa attend près de la porte. On rentre, Nino ? Oui. Le soir, le paillasson gratte de nouveau. Nino touche l'éclat de seau, un instant. Te voilà, Nino. Les bottes sont là. J'ai quelque chose, maintenant ! Nino avance trop vite vers le seau. Maman accroche le manteau.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Iris arrive en classe avec maman. Maman dit au revoir. Iris s'assoit sur le tapis. La maîtresse montre une coquille. Iris a une idée. Elle lève la main. Elle attend. Un camarade parle d'abord. Iris attend encore. &lt;emphasis&gt;puis&lt;/emphasis&gt; la maîtresse dit : Iris, c'est toi. Iris parle. Elle dit : la coquille est lisse. Le soir, maman demande. Iris dit : j'ai attendu. Puis j'ai parlé. [pause]</t>
+          <t>Le paillasson gratte sous les pieds. Des grains de sable restent dans les fibres. Ils piquent un peu, très fins. Un seau en fer est près des bottes. Sur le fer, un &lt;emphasis&gt;éclat de seau&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le seau ? Le seau sent le bord de mer. Les bottes sont rêches, un peu salées. Ça sent la mer. Tes mains sont froides, Nino. Je veux entendre la mer. Dans une coquille. On va à l'école. Le cartable est près de la porte. Oui, maman. Papa aide Nino à passer les bras. Le manteau sent un peu le sel. Je reviens te chercher. Oui, papa. Papa serre l'épaule de Nino. Ils poussent la porte de l'école. La classe sent les feuilles. Un tapis de laine attend sous la fenêtre. Bonjour. Bonjour, maîtresse. Nino pose le cartable près du tapis. Il s'assoit, le dos droit. La maîtresse pose une boîte sur la table. Elle ouvre le couvercle, sans un mot. Une coquille crème apparaît. Elle a des lignes, un peu rêche. La mer est dedans ! Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le dis, maintenant ! En ce moment, Nino ouvre la bouche. Ses mots se cognent à la classe. Un camarade parle près de la boîte. Personne ne tourne la tête. Oh. Le sourire de Nino disparaît. Ses épaules tombent un peu. Nino referme la bouche. Les mains restent sur les genoux. À la sortie, papa attend près de la porte. On rentre, Nino ? Oui. Le soir, le paillasson gratte de nouveau. Nino touche l'éclat de seau, un instant. Te voilà, Nino. Les bottes sont là. J'ai quelque chose, maintenant ! Nino avance trop vite vers le seau. Maman accroche le manteau. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>puis</t>
+          <t>éclat de seau</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,56 +1326,72 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_parler_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une coquille grince dans la poche de Nino.
-narrateur|Le bois du ponton est sombre, encore mouillé.
-narrateur|Ça sent le sel et les caisses de poisson.
-narrateur|Une écaille brille près d'une corde.
-narrateur|Les mouettes crient, très haut.
-papa|Tu as vu l'eau, Nino ?
-enfant-m|Elle tape le bois.
-papa|Elle est verte, ce soir.
-narrateur|Nino sort la coquille, toute rêche.
-enfant-m|Je veux que tu écoutes.
-enfant-m|La mer est dedans.
-papa|On l'écoute, alors.
-narrateur|En ce moment, papa compte des caisses.
-narrateur|Il parle vers le bout du ponton.
-narrateur|Sa voix se mêle aux mouettes.
-enfant-m|Papa, écoute !
-enfant-m|Hush, hush !
-narrateur|Les mots tombent dans les cris.
-narrateur|Personne ne se tourne.
-narrateur|La coquille reste froide dans la paume.
-enfant-m|Papa.
-narrateur|Papa compte encore, un doigt en l'air.
-narrateur|Nino ferme la bouche.
-narrateur|Il lève la main, tout droit.
-narrateur|La coquille est dans l'autre main.
-narrateur|Sa main reste en l'air, près de la corde.
-narrateur|Une mouette passe, puis s'éloigne.
-narrateur|Papa se tourne.
-papa|Tu voulais dire quelque chose ?
-enfant-m|La mer.
-enfant-m|Dans la coquille.
-papa|Je t'entends, maintenant.
-narrateur|Papa se baisse.
-narrateur|L'oreille touche le bord rêche.
-enfant-m|Hush.
-papa|Hush, oui.
-papa|Merci, Nino.
-papa|Tu as attendu, et je t'ai entendu.
-narrateur|L'eau tape encore le ponton, tout bas.
-narrateur|La coquille garde le même hush.
-papa|On la remet dans la poche ?
-enfant-m|Pour ce soir.</t>
+          <t>narrateur|Le paillasson gratte sous les pieds.
+narrateur|Des grains de sable restent dans les fibres.
+narrateur|Ils piquent un peu, très fins.
+narrateur|Un seau en fer est près des bottes.
+narrateur|Sur le fer, un éclat de seau luit.
+enfant-m|Il brille, papa.
+papa|Tu le vois, sur le seau ?
+narrateur|Le seau sent le bord de mer.
+narrateur|Les bottes sont rêches, un peu salées.
+enfant-m|Ça sent la mer.
+maman|Tes mains sont froides, Nino.
+enfant-m|Je veux entendre la mer.
+enfant-m|Dans une coquille.
+papa|On va à l'école.
+maman|Le cartable est près de la porte.
+enfant-m|Oui, maman.
+narrateur|Papa aide Nino à passer les bras.
+narrateur|Le manteau sent un peu le sel.
+papa|Je reviens te chercher.
+enfant-m|Oui, papa.
+narrateur|Papa serre l'épaule de Nino.
+narrateur|Ils poussent la porte de l'école.
+narrateur|La classe sent les feuilles.
+narrateur|Un tapis de laine attend sous la fenêtre.
+maitresse|Bonjour.
+enfant-m|Bonjour, maîtresse.
+narrateur|Nino pose le cartable près du tapis.
+narrateur|Il s'assoit, le dos droit.
+narrateur|La maîtresse pose une boîte sur la table.
+narrateur|Elle ouvre le couvercle, sans un mot.
+narrateur|Une coquille crème apparaît.
+narrateur|Elle a des lignes, un peu rêche.
+enfant-m|La mer est dedans !
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Je le dis, maintenant !
+narrateur|En ce moment, Nino ouvre la bouche.
+narrateur|Ses mots se cognent à la classe.
+narrateur|Un camarade parle près de la boîte.
+narrateur|Personne ne tourne la tête.
+enfant-m|Oh.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Ses épaules tombent un peu.
+narrateur|Nino referme la bouche.
+narrateur|Les mains restent sur les genoux.
+narrateur|À la sortie, papa attend près de la porte.
+papa|On rentre, Nino ?
+enfant-m|Oui.
+narrateur|Le soir, le paillasson gratte de nouveau.
+narrateur|Nino touche l'éclat de seau, un instant.
+maman|Te voilà, Nino.
+papa|Les bottes sont là.
+enfant-m|J'ai quelque chose, maintenant !
+narrateur|Nino avance trop vite vers le seau.
+narrateur|Maman accroche le manteau.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>radiateur,boite</t>
+          <t>seau,bottes</t>
         </is>
       </c>
     </row>
@@ -1407,12 +1423,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino veut parler. Que fait-il d'abord ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino veut &lt;emphasis level="moderate"&gt;parler&lt;/emphasis&gt;. Que fait-il d'abord ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Iris veut parler. Que fait-elle d'abord ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino veut &lt;emphasis&gt;parler&lt;/emphasis&gt;. Que fait-il d'abord ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1437,7 +1453,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Personne ne l'entend. Que fait Nino d'abord ?</t>
+          <t>Il lève la main et il attend. Que fait Nino ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1475,7 +1491,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1483,10 +1499,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1501,34 +1517,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>parler</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1537,23 +1557,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_leve_la_main_et_attend; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1586,17 +1606,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Ils s'assoient sur une caisse vide. Le bois est froid, un peu salé. Nino tend encore la coquille. Tu veux que j'écoute encore ? Oui. Papa écoute, longtemps. Tu m'as entendu. Oui. Quand les mouettes se sont tues un peu. Quand ta main était là. Une goutte tombe de la corde. Elle fait un rond dans l'eau verte. Elle est rêche, ta coquille ? Oui. Comme le bois. Nino la frotte contre sa manche. Un grain de sable tombe, tout fin. On la garde ? Dans la poche.</t>
+          <t>Nino parle trop vite, près du seau. Maman, la mer est dedans ! Maman n'a pas fini sa phrase. Le manteau est humide, Nino. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Il refuse de foncer. Nino referme la bouche. Il lève la main, près des bottes. Sa main reste en l'air. Maman finit d'accrocher le manteau. Nino garde la main haute. Tu veux venir près du seau ? Papa s'accroupit à la même hauteur. Nino pose un pied près du fer. Le seau est froid, un peu salé. La coquille est crème. La mer est peut-être dedans. On t'écoute. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Tu veux l'écouter ? Un peu, maman. La lumière touche le fer.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Ils s'assoient sur une caisse vide. Le bois est froid, un peu salé. Nino tend encore la coquille. Tu veux que j'écoute encore ? Oui. Papa écoute, longtemps. Tu m'as entendu. Oui. Quand les mouettes se sont tues un peu. Quand ta main était là. Une goutte tombe de la corde. Elle fait un rond dans l'eau verte. Elle est rêche, ta coquille ? Oui. Comme le bois. Nino la frotte contre sa manche. Un grain de sable tombe, tout fin. On la garde ? Dans la poche.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino parle trop vite, près du &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt;. Maman, la mer est dedans ! Maman n'a pas fini sa phrase. Le manteau est humide, Nino. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Il refuse de foncer. Nino referme la bouche. Il lève la main, près des bottes. Sa main reste en l'air. Maman finit d'accrocher le manteau. Nino garde la main haute. Tu veux venir près du seau ? Papa s'accroupit à la même hauteur. Nino pose un pied près du fer. Le seau est froid, un peu salé. La coquille est crème. La mer est peut-être dedans. On t'écoute. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Tu veux l'écouter ? Un peu, maman. La lumière touche le fer.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Iris a attendu. &lt;emphasis&gt;puis&lt;/emphasis&gt; elle a parlé. C'était son tour. [pause]</t>
+          <t>Nino parle trop vite, près du &lt;emphasis&gt;seau&lt;/emphasis&gt;. Maman, la mer est dedans ! Maman n'a pas fini sa phrase. Le manteau est humide, Nino. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Il refuse de foncer. Nino referme la bouche. Il lève la main, près des bottes. Sa main reste en l'air. Maman finit d'accrocher le manteau. Nino garde la main haute. Tu veux venir près du seau ? Papa s'accroupit à la même hauteur. Nino pose un pied près du fer. Le seau est froid, un peu salé. La coquille est crème. La mer est peut-être dedans. On t'écoute. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Tu veux l'écouter ? Un peu, maman. La lumière touche le fer. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1643,7 +1663,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1651,10 +1671,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1677,7 +1697,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>puis</t>
+          <t>seau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1691,16 +1711,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1709,10 +1729,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1725,30 +1745,43 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=la_porte_echoue_la_main_tient; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Ils s'assoient sur une caisse vide.
-narrateur|Le bois est froid, un peu salé.
-narrateur|Nino tend encore la coquille.
-papa|Tu veux que j'écoute encore ?
-enfant-m|Oui.
-narrateur|Papa écoute, longtemps.
-enfant-m|Tu m'as entendu.
-papa|Oui.
-papa|Quand les mouettes se sont tues un peu.
-papa|Quand ta main était là.
-narrateur|Une goutte tombe de la corde.
-narrateur|Elle fait un rond dans l'eau verte.
-papa|Elle est rêche, ta coquille ?
-enfant-m|Oui.
-enfant-m|Comme le bois.
-narrateur|Nino la frotte contre sa manche.
-narrateur|Un grain de sable tombe, tout fin.
-papa|On la garde ?
-enfant-m|Dans la poche.</t>
+          <t>narrateur|Nino parle trop vite, près du seau.
+enfant-m|Maman, la mer est dedans !
+narrateur|Maman n'a pas fini sa phrase.
+maman|Le manteau est humide, Nino.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Il refuse de foncer.
+narrateur|Nino referme la bouche.
+narrateur|Il lève la main, près des bottes.
+narrateur|Sa main reste en l'air.
+narrateur|Maman finit d'accrocher le manteau.
+narrateur|Nino garde la main haute.
+papa|Tu veux venir près du seau ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Nino pose un pied près du fer.
+narrateur|Le seau est froid, un peu salé.
+enfant-m|La coquille est crème.
+enfant-m|La mer est peut-être dedans.
+maman|On t'écoute.
+papa|Merci, Nino.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Nino se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu veux l'écouter ?
+enfant-m|Un peu, maman.
+narrateur|La lumière touche le fer.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>manteau,seau</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1808,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Le ponton sèche par plaques. Papa prend la main de Nino. On rentre ? Oui. Tu as entendu la mer. Oui. Je t'ai entendu, toi aussi. La coquille grince encore, tout bas. Les caisses restent alignées, mouillées. Elle est bien dans la poche ? Elle hush encore.</t>
+          <t>Nino prend la coquille trop vite. Je dis tout, d'un coup ! Le seau bascule d'un cran. Une botte glisse vers le paillasson. Oh. Nino avance les mains. Puis il s'arrête net. Attends, je regarde. Papa reste là, sans parler. Nino observe le fer, écoute la maison. Sur le seau, un éclat de seau luit. Là, près des bottes. Nino pose d'abord la coquille. Puis il redresse le seau. La mer, c'était trop vite. Tu veux l'écouter ici ? Oui, papa. Nino s'assoit près du seau. Mes mots se sont cognés. On est là. La lumière de l'entrée touche le fer. Nino pose la coquille contre l'oreille. Un hush arrive, un peu froid. Tu as fini ta phrase ? Presque.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Le ponton sèche par plaques. Papa prend la main de Nino. On rentre ? Oui. Tu as entendu la mer. Oui. Je t'ai entendu, toi aussi. La coquille grince encore, tout bas. Les caisses restent alignées, mouillées. Elle est bien dans la poche ? Elle hush encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino prend la coquille trop vite. Je dis tout, d'un coup ! Le seau bascule d'un cran. Une botte glisse vers le paillasson. Oh. Nino avance les mains. Puis il s'arrête net. Attends, je regarde. Papa reste là, sans parler. Nino observe le fer, écoute la maison. Sur le seau, un &lt;emphasis level="moderate"&gt;éclat de seau&lt;/emphasis&gt; luit. Là, près des bottes. Nino pose d'abord la coquille. Puis il redresse le seau. La mer, c'était trop vite. Tu veux l'écouter ici ? Oui, papa. Nino s'assoit près du seau. Mes mots se sont cognés. On est là. La lumière de l'entrée touche le fer. Nino pose la coquille contre l'oreille. Un hush arrive, un peu froid. Tu as fini ta phrase ? Presque.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Iris range son cartable. Maman l'attend près de la porte. [pause]</t>
+          <t>Nino prend la coquille trop vite. Je dis tout, d'un coup ! Le seau bascule d'un cran. Une botte glisse vers le paillasson. Oh. Nino avance les mains. Puis il s'arrête net. Attends, je regarde. Papa reste là, sans parler. Nino observe le fer, écoute la maison. Sur le seau, un &lt;emphasis&gt;éclat de seau&lt;/emphasis&gt; luit. Là, près des bottes. Nino pose d'abord la coquille. Puis il redresse le seau. La mer, c'était trop vite. Tu veux l'écouter ici ? Oui, papa. Nino s'assoit près du seau. Mes mots se sont cognés. On est là. La lumière de l'entrée touche le fer. Nino pose la coquille contre l'oreille. Un hush arrive, un peu froid. Tu as fini ta phrase ? Presque. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1832,7 +1865,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1840,10 +1873,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1864,28 +1897,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de seau</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1894,10 +1931,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1908,25 +1945,43 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sans_regarder_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Le ponton sèche par plaques.
-narrateur|Papa prend la main de Nino.
-papa|On rentre ?
-enfant-m|Oui.
-enfant-m|Tu as entendu la mer.
-papa|Oui.
-papa|Je t'ai entendu, toi aussi.
-narrateur|La coquille grince encore, tout bas.
-narrateur|Les caisses restent alignées, mouillées.
-papa|Elle est bien dans la poche ?
-enfant-m|Elle hush encore.</t>
+          <t>narrateur|Nino prend la coquille trop vite.
+enfant-m|Je dis tout, d'un coup !
+narrateur|Le seau bascule d'un cran.
+narrateur|Une botte glisse vers le paillasson.
+enfant-m|Oh.
+narrateur|Nino avance les mains.
+narrateur|Puis il s'arrête net.
+enfant-m|Attends, je regarde.
+narrateur|Papa reste là, sans parler.
+narrateur|Nino observe le fer, écoute la maison.
+narrateur|Sur le seau, un éclat de seau luit.
+enfant-m|Là, près des bottes.
+narrateur|Nino pose d'abord la coquille.
+narrateur|Puis il redresse le seau.
+enfant-m|La mer, c'était trop vite.
+papa|Tu veux l'écouter ici ?
+enfant-m|Oui, papa.
+narrateur|Nino s'assoit près du seau.
+enfant-m|Mes mots se sont cognés.
+maman|On est là.
+narrateur|La lumière de l'entrée touche le fer.
+narrateur|Nino pose la coquille contre l'oreille.
+narrateur|Un hush arrive, un peu froid.
+papa|Tu as fini ta phrase ?
+enfant-m|Presque.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>cartable,porte</t>
+          <t>bottes,coquille</t>
         </is>
       </c>
     </row>
@@ -1953,17 +2008,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La coquille hush dans la poche. Tu m'as entendu. Oui. Le sel colle encore aux doigts. Le ponton claque, tout doux.</t>
+          <t>Le seau brillait, papa. Tu le vois, comme ce matin ? Oui, sur le fer. Nino pose la coquille près du seau. On la laisse là ? Oui, maman. La lumière de l'entrée touche le fer. Nino pose la coquille contre son oreille. Un hush arrive, un peu salé. Je l'entends. Les bottes restent près du paillasson. Un éclat de seau reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La coquille hush dans la poche. Tu m'as entendu. Oui. Le sel colle encore aux doigts. Le ponton claque, tout doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau brillait, papa. Tu le vois, comme ce matin ? Oui, sur le fer. Nino pose la coquille près du seau. On la laisse là ? Oui, maman. La lumière de l'entrée touche le fer. Nino pose la coquille contre son oreille. Un hush arrive, un peu salé. Je l'entends. Les bottes restent près du paillasson. Un &lt;emphasis level="moderate"&gt;éclat de seau&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau brillait, papa. Tu le vois, comme ce matin ? Oui, sur le fer. Nino pose la coquille près du seau. On la laisse là ? Oui, maman. La lumière de l'entrée touche le fer. Nino pose la coquille contre son oreille. Un hush arrive, un peu salé. Je l'entends. Les bottes restent près du paillasson. Un &lt;emphasis&gt;éclat de seau&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2010,18 +2065,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2030,12 +2085,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2044,17 +2099,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de seau</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2063,11 +2122,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2076,28 +2135,44 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La coquille hush dans la poche.
-enfant-m|Tu m'as entendu.
-papa|Oui.
-narrateur|Le sel colle encore aux doigts.
-narrateur|Le ponton claque, tout doux.</t>
+          <t>enfant-m|Le seau brillait, papa.
+papa|Tu le vois, comme ce matin ?
+enfant-m|Oui, sur le fer.
+narrateur|Nino pose la coquille près du seau.
+maman|On la laisse là ?
+enfant-m|Oui, maman.
+narrateur|La lumière de l'entrée touche le fer.
+narrateur|Nino pose la coquille contre son oreille.
+narrateur|Un hush arrive, un peu salé.
+enfant-m|Je l'entends.
+narrateur|Les bottes restent près du paillasson.
+narrateur|Un éclat de seau reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>seau,coquille</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2210,6 +2285,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>